<commit_message>
Better list rendering (#138)
</commit_message>
<xml_diff>
--- a/src/ExcelsiorAspose.Tests/ComplexTypeWithCustomEnumerableRender.Null.verified.xlsx
+++ b/src/ExcelsiorAspose.Tests/ComplexTypeWithCustomEnumerableRender.Null.verified.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Name</t>
   </si>
@@ -26,9 +26,6 @@
   </si>
   <si>
     <t>John Doe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">● </t>
   </si>
 </sst>
 </file>
@@ -488,9 +485,7 @@
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
+      <c r="B2" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:B2"/>

</xml_diff>